<commit_message>
fix(exam-data): correct batch year typo for Agentic AI (AI4015)
The source xlsx (FSC!D14) had batch year '2022' for AI4015 Agentic
Artificial Intelligence, but this course is a 2023-batch CS elective.
Changed 2022 → 2023 in the source cell, then re-ran the transformation
pipeline.

Also fixed a course name typo in the same cell: 'Agentic Artificial
Intelligenc' → 'Agentic Artificial Intelligence' (missing trailing 'e').

Effect:
- AI4015 now appears for batch 2023 (CS, AI, DS departments) instead of 2022
- CS 2023 batch course count: 12 → 13 (Agentic AI added)
- Total entry count unchanged: 288
- No other courses affected

This is a one-off data integrity fix for a specific reported typo.
Any further source typos will be reported and fixed case-by-case.
</commit_message>
<xml_diff>
--- a/exam_schedule.xlsx
+++ b/exam_schedule.xlsx
@@ -3257,7 +3257,7 @@
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>Agentic Artificial Intelligenc</t>
+          <t>Agentic Artificial Intelligence</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>Agentic Artificial Intelligenc</t>
+          <t>Agentic Artificial Intelligence</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Agentic Artificial Intelligenc</t>
+          <t>Agentic Artificial Intelligence</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023</t>
         </is>
       </c>
     </row>

</xml_diff>